<commit_message>
feat: add enum_values column to command configuration
- Add '枚举取值说明' column (col 9) to command Excel
- Update CommandDef model with enum_values: dict[str,str]
- Update load_commands to parse new column via _parse_enum()
- Change _parse_enum() return type from dict[int,str] to dict[str,str]
  to support both integer keys (telemetry) and hex keys (commands)
- Update bitfield parser enum lookup to use str(raw_value)
- 30 commands now have enum values (AA AA:开/关, AA AA:使能/屏蔽, etc.)

Remote push requires network access. Run:
  git push --force origin master
</commit_message>
<xml_diff>
--- a/profiles/ppcu_rs422/commands/立即遥控指令配置表.xlsx
+++ b/profiles/ppcu_rs422/commands/立即遥控指令配置表.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Codex Workspace\02_Projects\项目文档\excel版遥测大表\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{543636CF-9CC4-4EEC-BC67-C70C17EDFCB4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1E49731-27D0-478C-A206-6DD1B0D50210}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="立即遥控指令" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="765" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="796" uniqueCount="368">
   <si>
     <t>序号</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1050,9 +1050,6 @@
     <t>TCHEDTTA115</t>
   </si>
   <si>
-    <t>请复位次数</t>
-  </si>
-  <si>
     <t>03 E1</t>
   </si>
   <si>
@@ -1158,6 +1155,37 @@
   </si>
   <si>
     <t>正常点火模式</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>枚举取值说明</t>
+  </si>
+  <si>
+    <t>AA AA:开;BB BB:关</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AA AA:主;BB BB:备</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AA AA:使能;BB BB:禁止</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AA AA:使能;BB BB:屏蔽</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AA AA:有效;BB BB:无效</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>AA AA:正常点火;BB BB:二次点火</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>清复位次数</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1165,7 +1193,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1214,6 +1242,13 @@
       <family val="2"/>
       <charset val="134"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -1233,7 +1268,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -1282,11 +1317,35 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD9D9D9"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1308,6 +1367,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1588,16 +1651,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H107"/>
+  <dimension ref="A1:I107"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="14.75" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="32" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.58203125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.08203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:9" ht="29" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1622,8 +1686,11 @@
       <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I1" s="9" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1631,7 +1698,7 @@
         <v>8</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D2" s="4" t="s">
         <v>10</v>
@@ -1647,7 +1714,7 @@
       </c>
       <c r="H2" s="5"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1673,7 +1740,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1699,7 +1766,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1723,7 +1790,7 @@
       </c>
       <c r="H5" s="5"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1747,7 +1814,7 @@
       </c>
       <c r="H6" s="5"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1771,7 +1838,7 @@
       </c>
       <c r="H7" s="5"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1797,7 +1864,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1821,7 +1888,7 @@
       </c>
       <c r="H9" s="5"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1845,7 +1912,7 @@
       </c>
       <c r="H10" s="5"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1871,7 +1938,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1879,7 +1946,7 @@
         <v>40</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D12" s="4" t="s">
         <v>10</v>
@@ -1897,7 +1964,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1923,7 +1990,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1949,7 +2016,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1975,7 +2042,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -2417,7 +2484,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -2443,7 +2510,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -2469,7 +2536,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -2495,7 +2562,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -2520,8 +2587,11 @@
       <c r="H36" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I36" s="10" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -2546,8 +2616,11 @@
       <c r="H37" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I37" s="10" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -2572,8 +2645,11 @@
       <c r="H38" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I38" s="10" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -2598,8 +2674,11 @@
       <c r="H39" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I39" s="10" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -2624,8 +2703,11 @@
       <c r="H40" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I40" s="10" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -2650,8 +2732,11 @@
       <c r="H41" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I41" s="10" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -2676,8 +2761,11 @@
       <c r="H42" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I42" s="10" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -2702,8 +2790,11 @@
       <c r="H43" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I43" s="10" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -2728,8 +2819,11 @@
       <c r="H44" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I44" s="10" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -2754,8 +2848,11 @@
       <c r="H45" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I45" s="10" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -2780,8 +2877,11 @@
       <c r="H46" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I46" s="10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -2806,8 +2906,11 @@
       <c r="H47" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I47" s="10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -2832,8 +2935,11 @@
       <c r="H48" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="49" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I48" s="10" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -2858,8 +2964,11 @@
       <c r="H49" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="50" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I49" s="10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>49</v>
       </c>
@@ -2884,8 +2993,11 @@
       <c r="H50" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="51" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I50" s="10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>50</v>
       </c>
@@ -2911,7 +3023,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="52" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>51</v>
       </c>
@@ -2936,8 +3048,11 @@
       <c r="H52" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="53" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I52" s="10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>52</v>
       </c>
@@ -2962,8 +3077,11 @@
       <c r="H53" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="54" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I53" s="10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>53</v>
       </c>
@@ -2988,8 +3106,11 @@
       <c r="H54" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="55" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I54" s="10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>54</v>
       </c>
@@ -3014,8 +3135,11 @@
       <c r="H55" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I55" s="10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>55</v>
       </c>
@@ -3040,8 +3164,11 @@
       <c r="H56" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I56" s="10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>56</v>
       </c>
@@ -3066,8 +3193,11 @@
       <c r="H57" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I57" s="10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>57</v>
       </c>
@@ -3092,8 +3222,11 @@
       <c r="H58" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I58" s="10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>58</v>
       </c>
@@ -3118,8 +3251,11 @@
       <c r="H59" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I59" s="10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>59</v>
       </c>
@@ -3144,8 +3280,11 @@
       <c r="H60" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I60" s="10" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>60</v>
       </c>
@@ -3170,8 +3309,11 @@
       <c r="H61" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I61" s="10" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>61</v>
       </c>
@@ -3196,8 +3338,11 @@
       <c r="H62" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I62" s="10" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>62</v>
       </c>
@@ -3222,8 +3367,9 @@
       <c r="H63" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I63" s="10"/>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>63</v>
       </c>
@@ -3248,8 +3394,11 @@
       <c r="H64" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I64" s="10" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>64</v>
       </c>
@@ -3275,7 +3424,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>65</v>
       </c>
@@ -3301,7 +3450,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="67" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>66</v>
       </c>
@@ -3327,7 +3476,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>67</v>
       </c>
@@ -3353,7 +3502,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>68</v>
       </c>
@@ -3378,8 +3527,11 @@
       <c r="H69" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I69" s="10" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>69</v>
       </c>
@@ -3405,7 +3557,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>70</v>
       </c>
@@ -3431,7 +3583,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>71</v>
       </c>
@@ -3457,7 +3609,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>72</v>
       </c>
@@ -3483,7 +3635,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>73</v>
       </c>
@@ -3508,8 +3660,11 @@
       <c r="H74" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I74" s="10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>74</v>
       </c>
@@ -3535,7 +3690,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>75</v>
       </c>
@@ -3561,7 +3716,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>76</v>
       </c>
@@ -3587,7 +3742,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>77</v>
       </c>
@@ -3613,7 +3768,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="79" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>78</v>
       </c>
@@ -3639,7 +3794,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="80" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>79</v>
       </c>
@@ -4081,7 +4236,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="97" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>96</v>
       </c>
@@ -4107,7 +4262,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="98" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>97</v>
       </c>
@@ -4133,7 +4288,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="99" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>98</v>
       </c>
@@ -4159,7 +4314,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="100" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>99</v>
       </c>
@@ -4185,7 +4340,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="101" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>100</v>
       </c>
@@ -4211,7 +4366,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="102" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>101</v>
       </c>
@@ -4237,7 +4392,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="103" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>102</v>
       </c>
@@ -4263,7 +4418,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="104" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>103</v>
       </c>
@@ -4289,7 +4444,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="105" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>104</v>
       </c>
@@ -4314,8 +4469,11 @@
       <c r="H105" s="5" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="106" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="I105" s="10" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>105</v>
       </c>
@@ -4323,45 +4481,45 @@
         <v>327</v>
       </c>
       <c r="C106" s="4" t="s">
+        <v>367</v>
+      </c>
+      <c r="D106" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E106" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F106" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="G106" s="4" t="s">
         <v>328</v>
-      </c>
-      <c r="D106" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E106" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F106" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="G106" s="4" t="s">
-        <v>329</v>
       </c>
       <c r="H106" s="5" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="107" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>106</v>
       </c>
       <c r="B107" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="C107" s="4" t="s">
         <v>330</v>
       </c>
-      <c r="C107" s="4" t="s">
+      <c r="D107" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E107" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F107" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="G107" s="4" t="s">
         <v>331</v>
-      </c>
-      <c r="D107" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E107" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F107" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="G107" s="4" t="s">
-        <v>332</v>
       </c>
       <c r="H107" s="5" t="s">
         <v>102</v>
@@ -4387,45 +4545,45 @@
   <sheetData>
     <row r="1" spans="1:7" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A1" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>333</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="C1" s="6" t="s">
         <v>334</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="D1" s="6" t="s">
         <v>335</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="E1" s="7" t="s">
         <v>336</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="F1" s="7" t="s">
         <v>337</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="G1" s="6" t="s">
         <v>338</v>
-      </c>
-      <c r="G1" s="6" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="8" t="s">
+        <v>339</v>
+      </c>
+      <c r="B2" s="8" t="s">
         <v>340</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="C2" s="8" t="s">
         <v>341</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="D2" s="8" t="s">
         <v>342</v>
       </c>
-      <c r="D2" s="8" t="s">
+      <c r="E2" s="8" t="s">
         <v>343</v>
       </c>
-      <c r="E2" s="8" t="s">
+      <c r="F2" s="8" t="s">
         <v>344</v>
-      </c>
-      <c r="F2" s="8" t="s">
-        <v>345</v>
       </c>
       <c r="G2" s="8"/>
     </row>
@@ -4433,16 +4591,16 @@
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8" t="s">
+        <v>345</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>342</v>
+      </c>
+      <c r="E3" s="8" t="s">
         <v>346</v>
       </c>
-      <c r="D3" s="8" t="s">
-        <v>343</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>347</v>
-      </c>
       <c r="F3" s="8" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="G3" s="8"/>
     </row>
@@ -4450,24 +4608,24 @@
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D4" s="8">
         <v>2</v>
       </c>
       <c r="E4" s="8" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="F4" s="8" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="G4" s="8"/>
     </row>
-    <row r="5" spans="1:7" ht="28" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D5" s="8">
         <v>14</v>
@@ -4476,54 +4634,54 @@
         <v>0</v>
       </c>
       <c r="F5" s="8" t="s">
+        <v>350</v>
+      </c>
+      <c r="G5" s="8" t="s">
         <v>351</v>
       </c>
-      <c r="G5" s="8" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="28" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8" t="s">
+        <v>352</v>
+      </c>
+      <c r="D6" s="8" t="s">
+        <v>342</v>
+      </c>
+      <c r="F6" s="8" t="s">
         <v>353</v>
       </c>
-      <c r="D6" s="8" t="s">
-        <v>343</v>
-      </c>
-      <c r="F6" s="8" t="s">
+      <c r="G6" s="8" t="s">
         <v>354</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>
       <c r="F7" s="8"/>
       <c r="G7" s="8"/>
     </row>
-    <row r="8" spans="1:7" ht="112" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" ht="42" x14ac:dyDescent="0.3">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
       <c r="G8" s="8" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
   </sheetData>

</xml_diff>